<commit_message>
Fixed typo in PUSH Ra STEP numbering
</commit_message>
<xml_diff>
--- a/CPU Design/L1IsSequences.xlsx
+++ b/CPU Design/L1IsSequences.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Original" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'+Address bus'!$A$1:$AL$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'+Address bus'!$J$1:$J$176</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
@@ -9962,7 +9962,7 @@
         <v>8</v>
       </c>
       <c r="C87">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E87" s="5" t="s">
         <v>21</v>
@@ -10057,7 +10057,7 @@
         <v>8</v>
       </c>
       <c r="C88">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E88" s="5" t="s">
         <v>21</v>
@@ -10155,7 +10155,7 @@
         <v>8</v>
       </c>
       <c r="C89">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E89" s="5" t="s">
         <v>21</v>
@@ -10253,7 +10253,7 @@
         <v>8</v>
       </c>
       <c r="C90">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>21</v>
@@ -10348,7 +10348,7 @@
         <v>8</v>
       </c>
       <c r="C91">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E91" s="5" t="s">
         <v>21</v>
@@ -10446,7 +10446,7 @@
         <v>8</v>
       </c>
       <c r="C92">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E92" s="5" t="s">
         <v>21</v>
@@ -10544,7 +10544,7 @@
         <v>8</v>
       </c>
       <c r="C93">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E93" s="5" t="s">
         <v>21</v>
@@ -10639,7 +10639,7 @@
         <v>8</v>
       </c>
       <c r="C94">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E94" s="5" t="s">
         <v>21</v>
@@ -10737,7 +10737,7 @@
         <v>8</v>
       </c>
       <c r="C95">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>21</v>
@@ -10835,7 +10835,7 @@
         <v>8</v>
       </c>
       <c r="C96">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E96" s="5" t="s">
         <v>21</v>
@@ -10933,7 +10933,7 @@
         <v>8</v>
       </c>
       <c r="C97">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>21</v>
@@ -11031,7 +11031,7 @@
         <v>8</v>
       </c>
       <c r="C98">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>21</v>
@@ -11129,7 +11129,7 @@
         <v>8</v>
       </c>
       <c r="C99">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>21</v>
@@ -11227,7 +11227,7 @@
         <v>8</v>
       </c>
       <c r="C100">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E100" s="5" t="s">
         <v>21</v>
@@ -11325,7 +11325,7 @@
         <v>8</v>
       </c>
       <c r="C101">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>21</v>
@@ -11423,7 +11423,7 @@
         <v>8</v>
       </c>
       <c r="C102">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E102" s="4" t="s">
         <v>24</v>

</xml_diff>